<commit_message>
demo: add oncho forms
</commit_message>
<xml_diff>
--- a/Demo/ONCHO/epi/demo_oncho_epi_9999_3_ov16.xlsx
+++ b/Demo/ONCHO/epi/demo_oncho_epi_9999_3_ov16.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\ONCHO\epi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B1AFA6-8739-48D4-B340-1DF4F98BC640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE591EE-2360-4A82-9E2B-1EC2C1412CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -327,9 +327,6 @@
     <t>OV16 test result</t>
   </si>
   <si>
-    <t>Enter batch number</t>
-  </si>
-  <si>
     <t>d_OV16_result</t>
   </si>
   <si>
@@ -387,9 +384,6 @@
     <t>d9999</t>
   </si>
   <si>
-    <t>Results FTS</t>
-  </si>
-  <si>
     <t>d_code_id1</t>
   </si>
   <si>
@@ -496,6 +490,12 @@
   </si>
   <si>
     <t>d_Notes</t>
+  </si>
+  <si>
+    <t>Results OV16</t>
+  </si>
+  <si>
+    <t>Enter lot number</t>
   </si>
 </sst>
 </file>
@@ -1166,10 +1166,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="39" t="s">
         <v>106</v>
-      </c>
-      <c r="C3" s="39" t="s">
-        <v>107</v>
       </c>
       <c r="D3" s="39"/>
       <c r="E3" s="24"/>
@@ -1196,10 +1196,10 @@
         <v>15</v>
       </c>
       <c r="B4" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="39" t="s">
         <v>108</v>
-      </c>
-      <c r="C4" s="39" t="s">
-        <v>109</v>
       </c>
       <c r="D4" s="39"/>
       <c r="E4" s="24"/>
@@ -1217,7 +1217,7 @@
         <v>80</v>
       </c>
       <c r="O4" s="23" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P4" s="23"/>
       <c r="Q4" s="23"/>
@@ -1228,10 +1228,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="39" t="s">
         <v>111</v>
-      </c>
-      <c r="C5" s="39" t="s">
-        <v>112</v>
       </c>
       <c r="D5" s="39"/>
       <c r="E5" s="24"/>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="O5" s="23"/>
       <c r="P5" s="23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Q5" s="23"/>
       <c r="R5" s="23"/>
@@ -1260,10 +1260,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="39" t="s">
         <v>114</v>
-      </c>
-      <c r="C6" s="39" t="s">
-        <v>115</v>
       </c>
       <c r="D6" s="39"/>
       <c r="E6" s="24"/>
@@ -1283,7 +1283,7 @@
       <c r="O6" s="23"/>
       <c r="P6" s="23"/>
       <c r="Q6" s="23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R6" s="23"/>
     </row>
@@ -1309,13 +1309,13 @@
     </row>
     <row r="8" spans="1:18" s="9" customFormat="1" ht="63">
       <c r="A8" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="C8" s="39" t="s">
         <v>118</v>
-      </c>
-      <c r="C8" s="39" t="s">
-        <v>119</v>
       </c>
       <c r="D8" s="39"/>
       <c r="E8" s="24"/>
@@ -1416,10 +1416,10 @@
         <v>63</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>121</v>
+        <v>156</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="19"/>
@@ -1518,17 +1518,17 @@
         <v>15</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D16" s="29"/>
       <c r="E16" s="28"/>
       <c r="F16" s="28"/>
       <c r="G16" s="28"/>
       <c r="H16" s="29" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I16" s="28"/>
       <c r="J16" s="29"/>
@@ -1542,7 +1542,7 @@
       <c r="P16" s="23"/>
       <c r="Q16" s="23"/>
       <c r="R16" s="30" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:20" s="9" customFormat="1">
@@ -1569,20 +1569,20 @@
     </row>
     <row r="18" spans="1:20" s="9" customFormat="1">
       <c r="A18" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" s="31" t="s">
         <v>126</v>
-      </c>
-      <c r="B18" s="31" t="s">
-        <v>127</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>128</v>
       </c>
       <c r="D18" s="31"/>
       <c r="E18" s="31"/>
       <c r="F18" s="31"/>
       <c r="G18" s="31"/>
       <c r="H18" s="31" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I18" s="31"/>
       <c r="J18" s="31" t="s">
@@ -1601,20 +1601,20 @@
     </row>
     <row r="19" spans="1:20" s="9" customFormat="1" ht="31.5">
       <c r="A19" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>129</v>
+      </c>
+      <c r="C19" s="32" t="s">
         <v>130</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>131</v>
-      </c>
-      <c r="C19" s="32" t="s">
-        <v>132</v>
       </c>
       <c r="D19" s="32"/>
       <c r="E19" s="31"/>
       <c r="F19" s="33"/>
       <c r="G19" s="34"/>
       <c r="H19" s="32" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I19" s="31"/>
       <c r="J19" s="31" t="s">
@@ -1636,17 +1636,17 @@
         <v>21</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C20" s="32" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D20" s="32"/>
       <c r="E20" s="31"/>
       <c r="F20" s="33"/>
       <c r="G20" s="34"/>
       <c r="H20" s="32" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I20" s="31"/>
       <c r="J20" s="31" t="s">
@@ -1668,21 +1668,21 @@
         <v>21</v>
       </c>
       <c r="B21" s="32" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C21" s="32" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D21" s="32"/>
       <c r="E21" s="31"/>
       <c r="F21" s="33" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G21" s="34" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I21" s="31"/>
       <c r="J21" s="31" t="s">
@@ -1729,7 +1729,7 @@
         <v>17</v>
       </c>
       <c r="C23" s="36" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D23" s="36"/>
       <c r="E23" s="35"/>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="H23" s="36"/>
       <c r="I23" s="35" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J23" s="36" t="s">
         <v>14</v>
@@ -1787,7 +1787,7 @@
         <v>16</v>
       </c>
       <c r="C25" s="39" t="s">
-        <v>101</v>
+        <v>157</v>
       </c>
       <c r="D25" s="39"/>
       <c r="E25" s="24"/>
@@ -1812,7 +1812,7 @@
         <v>18</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C26" s="39" t="s">
         <v>100</v>
@@ -1840,7 +1840,7 @@
         <v>19</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C27" s="39" t="s">
         <v>20</v>
@@ -1850,7 +1850,7 @@
       <c r="F27" s="23"/>
       <c r="G27" s="40"/>
       <c r="H27" s="23" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I27" s="23"/>
       <c r="J27" s="24" t="s">
@@ -1870,7 +1870,7 @@
         <v>15</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C28" s="39" t="s">
         <v>20</v>
@@ -1880,7 +1880,7 @@
       <c r="F28" s="23"/>
       <c r="G28" s="40"/>
       <c r="H28" s="24" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="I28" s="23"/>
       <c r="J28" s="24" t="s">
@@ -1900,7 +1900,7 @@
         <v>21</v>
       </c>
       <c r="B29" s="24" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C29" s="39" t="s">
         <v>22</v>
@@ -1968,7 +1968,7 @@
         <v>23</v>
       </c>
       <c r="B32" s="24" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C32" s="39"/>
       <c r="D32" s="39"/>
@@ -1992,7 +1992,7 @@
         <v>24</v>
       </c>
       <c r="B33" s="41" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C33" s="42"/>
       <c r="D33" s="42"/>
@@ -2384,24 +2384,24 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>143</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -2417,24 +2417,24 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>148</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -2470,7 +2470,7 @@
         <v>99</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
         <v>55</v>

</xml_diff>